<commit_message>
Added images and documentation draft
</commit_message>
<xml_diff>
--- a/EXCEL FILEOVI/ZAVRSNI EXCEL - SIM RESULTS .xlsx
+++ b/EXCEL FILEOVI/ZAVRSNI EXCEL - SIM RESULTS .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/523341E057C2D1B5/Documents/2526 - LJETNI SEMESTAR/Bachelor-Thesis/EXCEL FILEOVI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2055" documentId="8_{749E225B-507B-4645-922D-F24EE2B83FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94C9D64A-A2CF-4231-925A-18DBFBDA2286}"/>
+  <xr:revisionPtr revIDLastSave="2080" documentId="8_{749E225B-507B-4645-922D-F24EE2B83FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4DF8B01-B38E-4E7D-99DA-CA18E4678049}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="4" xr2:uid="{5A5A50C3-7C6B-466F-847F-D23E3D13151B}"/>
+    <workbookView xWindow="8370" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{5A5A50C3-7C6B-466F-847F-D23E3D13151B}"/>
   </bookViews>
   <sheets>
     <sheet name="SZE SIM RESULTS" sheetId="1" r:id="rId1"/>
@@ -184,8 +184,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -276,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -293,6 +294,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5160,15 +5169,6 @@
     <row r="90" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="K17:N17"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="K49:N49"/>
-    <mergeCell ref="K65:N65"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A49:D49"/>
-    <mergeCell ref="A65:D65"/>
     <mergeCell ref="P65:S65"/>
     <mergeCell ref="U65:X65"/>
     <mergeCell ref="F1:I1"/>
@@ -5185,6 +5185,15 @@
     <mergeCell ref="U17:X17"/>
     <mergeCell ref="U33:X33"/>
     <mergeCell ref="K1:N1"/>
+    <mergeCell ref="K17:N17"/>
+    <mergeCell ref="K33:N33"/>
+    <mergeCell ref="K49:N49"/>
+    <mergeCell ref="K65:N65"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A65:D65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5196,24 +5205,24 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.59765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.59765625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.59765625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.6640625" customWidth="1"/>
     <col min="16" max="16" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.19921875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="6.265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.59765625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="14.3984375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11.73046875" bestFit="1" customWidth="1"/>
@@ -5319,70 +5328,70 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="9">
         <v>4.7282000000000002</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="9">
         <f>10^(B3/20)</f>
         <v>1.7234948895886821</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="9">
         <f>C3^2</f>
         <v>2.9704346344383037</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="9">
         <v>8.2105440000000005</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="9">
         <f>10^(G3/20)</f>
         <v>2.5735179396168371</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="9">
         <f>H3^2</f>
         <v>6.6229945855296899</v>
       </c>
       <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="9">
         <v>10.579746999999999</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="9">
         <f>10^(L3/20)</f>
         <v>3.3805498929777942</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="9">
         <f>M3^2</f>
         <v>11.428117578912175</v>
       </c>
       <c r="P3" s="1">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="11">
         <v>11.47996</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="11">
         <f>10^(Q3/20)</f>
         <v>3.7497127543496922</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="11">
         <f>R3^2</f>
         <v>14.060345740132755</v>
       </c>
       <c r="U3" s="1">
         <v>1</v>
       </c>
-      <c r="V3" s="2">
+      <c r="V3" s="9">
         <v>11.932463</v>
       </c>
-      <c r="W3" s="2">
+      <c r="W3" s="9">
         <f>10^(V3/20)</f>
         <v>3.950236977136218</v>
       </c>
-      <c r="X3" s="2">
+      <c r="X3" s="9">
         <f>W3^2</f>
         <v>15.604372175534285</v>
       </c>
@@ -5391,70 +5400,70 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="9">
         <v>-2.4359999999999999</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="9">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
         <v>0.75544004056761893</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="9">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
         <v>0.57068965489280576</v>
       </c>
       <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="9">
         <v>-2.1788400000000001</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="9">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
         <v>0.77814046470960674</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="9">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
         <v>0.60550258281848268</v>
       </c>
       <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="9">
         <v>-4.9427500000000002</v>
       </c>
-      <c r="M4" s="2">
+      <c r="M4" s="9">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
         <v>0.56606004296981571</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="9">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
         <v>0.3204239722469896</v>
       </c>
       <c r="P4" s="1">
         <v>2</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="11">
         <v>-8.2892419999999998</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="11">
         <f t="shared" ref="R4:R8" si="6">10^(Q4/20)</f>
         <v>0.38506841735340325</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="11">
         <f t="shared" ref="S4:S10" si="7">R4^2</f>
         <v>0.14827768604305475</v>
       </c>
       <c r="U4" s="1">
         <v>2</v>
       </c>
-      <c r="V4" s="2">
+      <c r="V4" s="9">
         <v>-11.64531</v>
       </c>
-      <c r="W4" s="2">
+      <c r="W4" s="9">
         <f t="shared" ref="W4:W10" si="8">10^(V4/20)</f>
         <v>0.26165829069454205</v>
       </c>
-      <c r="X4" s="2">
+      <c r="X4" s="9">
         <f t="shared" ref="X4:X10" si="9">W4^2</f>
         <v>6.8465061089189469E-2</v>
       </c>
@@ -5463,70 +5472,70 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="9">
         <v>-22.338000000000001</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="9">
         <f t="shared" si="0"/>
         <v>7.6401168351701826E-2</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="9">
         <f t="shared" si="1"/>
         <v>5.8371385255050843E-3</v>
       </c>
       <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="9">
         <v>-14.470370000000001</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="9">
         <f t="shared" si="2"/>
         <v>0.18900857159329354</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="9">
         <f t="shared" si="3"/>
         <v>3.5724240135737169E-2</v>
       </c>
       <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="9">
         <v>-10.854979999999999</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="9">
         <f t="shared" si="4"/>
         <v>0.28658337967398984</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="9">
         <f t="shared" si="5"/>
         <v>8.2130033505366212E-2</v>
       </c>
       <c r="P5" s="1">
         <v>3</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="11">
         <v>-12.060734999999999</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="11">
         <f t="shared" si="6"/>
         <v>0.249438364326283</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="11">
         <f t="shared" si="7"/>
         <v>6.2219497597771491E-2</v>
       </c>
       <c r="U5" s="1">
         <v>3</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="9">
         <v>-14.34806</v>
       </c>
-      <c r="W5" s="2">
+      <c r="W5" s="9">
         <f t="shared" si="8"/>
         <v>0.19168891535642241</v>
       </c>
-      <c r="X5" s="2">
+      <c r="X5" s="9">
         <f t="shared" si="9"/>
         <v>3.6744640270521677E-2</v>
       </c>
@@ -5535,70 +5544,70 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="9">
         <v>-15.955</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="9">
         <f t="shared" si="0"/>
         <v>0.1593125539925771</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="9">
         <f t="shared" si="1"/>
         <v>2.5380489859637794E-2</v>
       </c>
       <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="9">
         <v>-19.469000000000001</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="9">
         <f t="shared" si="2"/>
         <v>0.10630409633445624</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="9">
         <f t="shared" si="3"/>
         <v>1.1300560897485353E-2</v>
       </c>
       <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="9">
         <v>-24.02542</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="9">
         <f t="shared" si="4"/>
         <v>6.2911349317847601E-2</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="9">
         <f t="shared" si="5"/>
         <v>3.9578378729922441E-3</v>
       </c>
       <c r="P6" s="1">
         <v>4</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="11">
         <v>-18.432680000000001</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="11">
         <f t="shared" si="6"/>
         <v>0.11977495048699868</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="11">
         <f t="shared" si="7"/>
         <v>1.4346038764162987E-2</v>
       </c>
       <c r="U6" s="1">
         <v>4</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="9">
         <v>-18.438700000000001</v>
       </c>
-      <c r="W6" s="2">
+      <c r="W6" s="9">
         <f t="shared" si="8"/>
         <v>0.11969196585107088</v>
       </c>
-      <c r="X6" s="2">
+      <c r="X6" s="9">
         <f t="shared" si="9"/>
         <v>1.4326166689293917E-2</v>
       </c>
@@ -5607,70 +5616,70 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="9">
         <v>-31.186</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="9">
         <f t="shared" si="0"/>
         <v>2.7586715750763942E-2</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="9">
         <f t="shared" si="1"/>
         <v>7.6102688591344735E-4</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="9">
         <v>-20.594619999999999</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="9">
         <f t="shared" si="2"/>
         <v>9.3383253326739343E-2</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="9">
         <f t="shared" si="3"/>
         <v>8.7204320018859742E-3</v>
       </c>
       <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="9">
         <v>-25.769276999999999</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="9">
         <f t="shared" si="4"/>
         <v>5.1467864628410208E-2</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="9">
         <f t="shared" si="5"/>
         <v>2.6489410894083585E-3</v>
       </c>
       <c r="P7" s="1">
         <v>5</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="11">
         <v>-32.445210000000003</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="11">
         <f t="shared" si="6"/>
         <v>2.3863794472581724E-2</v>
       </c>
-      <c r="S7" s="2">
+      <c r="S7" s="11">
         <f t="shared" si="7"/>
         <v>5.6948068662962211E-4</v>
       </c>
       <c r="U7" s="1">
         <v>5</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="9">
         <v>-24.84498</v>
       </c>
-      <c r="W7" s="2">
+      <c r="W7" s="9">
         <f t="shared" si="8"/>
         <v>5.7246771612448344E-2</v>
       </c>
-      <c r="X7" s="2">
+      <c r="X7" s="9">
         <f t="shared" si="9"/>
         <v>3.2771928600478215E-3</v>
       </c>
@@ -5679,70 +5688,70 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="9">
         <v>-23.439900000000002</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="9">
         <f t="shared" si="0"/>
         <v>6.7298440425900177E-2</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="9">
         <f t="shared" si="1"/>
         <v>4.5290800837584355E-3</v>
       </c>
       <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="9">
         <v>-35.854080000000003</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="9">
         <f t="shared" si="2"/>
         <v>1.611743769355151E-2</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="9">
         <f t="shared" si="3"/>
         <v>2.5977179780551501E-4</v>
       </c>
       <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="9">
         <v>-23.938179999999999</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="9">
         <f t="shared" si="4"/>
         <v>6.3546407002131045E-2</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="9">
         <f t="shared" si="5"/>
         <v>4.0381458428804893E-3</v>
       </c>
       <c r="P8" s="1">
         <v>6</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="11">
         <v>-31.05416</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="11">
         <f t="shared" si="6"/>
         <v>2.8008638610887291E-2</v>
       </c>
-      <c r="S8" s="2">
+      <c r="S8" s="11">
         <f t="shared" si="7"/>
         <v>7.8448383683528639E-4</v>
       </c>
       <c r="U8" s="1">
         <v>6</v>
       </c>
-      <c r="V8" s="2">
+      <c r="V8" s="9">
         <v>-38.838008000000002</v>
       </c>
-      <c r="W8" s="2">
+      <c r="W8" s="9">
         <f>10^(V8/20)</f>
         <v>1.1431404696791313E-2</v>
       </c>
-      <c r="X8" s="2">
+      <c r="X8" s="9">
         <f t="shared" si="9"/>
         <v>1.3067701334182249E-4</v>
       </c>
@@ -5751,70 +5760,70 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="9">
         <v>-36.588999999999999</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="9">
         <f t="shared" si="0"/>
         <v>1.4809827498930051E-2</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="9">
         <f t="shared" si="1"/>
         <v>2.1933099054806474E-4</v>
       </c>
       <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="9">
         <v>-25.92764</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="9">
         <f t="shared" si="2"/>
         <v>5.0537994056481295E-2</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="9">
         <f t="shared" si="3"/>
         <v>2.5540888432529388E-3</v>
       </c>
       <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="9">
         <v>-32.496220000000001</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="9">
         <f t="shared" si="4"/>
         <v>2.3724059250121266E-2</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="9">
         <f t="shared" si="5"/>
         <v>5.6283098730326438E-4</v>
       </c>
       <c r="P9" s="1">
         <v>7</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="11">
         <v>-28.146439999999998</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="11">
         <f>10^(Q9/20)</f>
         <v>3.9145153463563898E-2</v>
       </c>
-      <c r="S9" s="2">
+      <c r="S9" s="11">
         <f t="shared" si="7"/>
         <v>1.5323430396859685E-3</v>
       </c>
       <c r="U9" s="1">
         <v>7</v>
       </c>
-      <c r="V9" s="2">
+      <c r="V9" s="9">
         <v>-36.419750000000001</v>
       </c>
-      <c r="W9" s="2">
+      <c r="W9" s="9">
         <f>10^(V9/20)</f>
         <v>1.5101236183902978E-2</v>
       </c>
-      <c r="X9" s="2">
+      <c r="X9" s="9">
         <f t="shared" si="9"/>
         <v>2.280473342820206E-4</v>
       </c>
@@ -5823,70 +5832,70 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="9">
         <v>-28.710799999999999</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="9">
         <f t="shared" si="0"/>
         <v>3.6682590697079062E-2</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="9">
         <f t="shared" si="1"/>
         <v>1.3456124602494314E-3</v>
       </c>
       <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="9">
         <v>-38.089199999999998</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="9">
         <f t="shared" si="2"/>
         <v>1.2460629986291331E-2</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="9">
         <f t="shared" si="3"/>
         <v>1.5526729965526268E-4</v>
       </c>
       <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="9">
         <v>-35.921900000000001</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="9">
         <f t="shared" si="4"/>
         <v>1.5992081706261624E-2</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="9">
         <f t="shared" si="5"/>
         <v>2.557466772997477E-4</v>
       </c>
       <c r="P10" s="1">
         <v>8</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="11">
         <v>-32.048209999999997</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="11">
         <f>10^(Q10/20)</f>
         <v>2.4979831238876763E-2</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="11">
         <f t="shared" si="7"/>
         <v>6.2399196872276342E-4</v>
       </c>
       <c r="U10" s="1">
         <v>8</v>
       </c>
-      <c r="V10" s="2">
+      <c r="V10" s="9">
         <v>-32.489280000000001</v>
       </c>
-      <c r="W10" s="2">
+      <c r="W10" s="9">
         <f t="shared" si="8"/>
         <v>2.3743022277629328E-2</v>
       </c>
-      <c r="X10" s="2">
+      <c r="X10" s="9">
         <f t="shared" si="9"/>
         <v>5.6373110687600256E-4</v>
       </c>
@@ -5895,226 +5904,226 @@
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="9">
         <f>SQRT(SUM(D4:D10)/D3)</f>
         <v>0.45270353589867951</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
       <c r="F11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="9">
         <f>SQRT(SUM(I4:I10)/I3)</f>
         <v>0.3166852054852487</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
       <c r="K11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L11" s="9">
         <f>SQRT(SUM(N4:N10)/N3)</f>
         <v>0.19033646694474435</v>
       </c>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
       <c r="P11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="11">
         <f>SQRT(SUM(S4:S10)/S3)</f>
         <v>0.1274400276729003</v>
       </c>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
       <c r="U11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="V11" s="2">
+      <c r="V11" s="9">
         <f>SQRT(SUM(X4:X10)/X3)</f>
         <v>8.904797288767928E-2</v>
       </c>
-      <c r="W11" s="1"/>
-      <c r="X11" s="1"/>
+      <c r="W11" s="9"/>
+      <c r="X11" s="9"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="10">
         <f>B11*100</f>
         <v>45.270353589867952</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
       <c r="F12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="10">
         <f>G11*100</f>
         <v>31.668520548524871</v>
       </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
       <c r="K12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="10">
         <f>L11*100</f>
         <v>19.033646694474434</v>
       </c>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
       <c r="P12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="Q12" s="4">
+      <c r="Q12" s="12">
         <f>Q11*100</f>
         <v>12.744002767290031</v>
       </c>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="11"/>
       <c r="U12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="V12" s="4">
+      <c r="V12" s="10">
         <f>V11*100</f>
         <v>8.9047972887679272</v>
       </c>
-      <c r="W12" s="1"/>
-      <c r="X12" s="1"/>
+      <c r="W12" s="9"/>
+      <c r="X12" s="9"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="9">
         <v>14.321999999999999</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
       <c r="F13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="9">
         <v>14.577999999999999</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
       <c r="K13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="9">
         <v>11.843</v>
       </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
       <c r="P13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="11">
         <v>9.5259999999999998</v>
       </c>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
       <c r="U13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="V13" s="1">
+      <c r="V13" s="9">
         <v>7.8639000000000001</v>
       </c>
-      <c r="W13" s="1"/>
-      <c r="X13" s="1"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="9">
         <v>116.68</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
       <c r="F14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="9">
         <v>113.01</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
       <c r="K14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="9">
         <v>109.43</v>
       </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
       <c r="P14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="11">
         <v>107.89</v>
       </c>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
       <c r="U14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V14" s="1">
+      <c r="V14" s="9">
         <v>107.12</v>
       </c>
-      <c r="W14" s="1"/>
-      <c r="X14" s="1"/>
+      <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="10">
         <f>(B13/B14)*100</f>
         <v>12.274597188892697</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
       <c r="F15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="10">
         <f>(G13/G14)*100</f>
         <v>12.899743385541102</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
       <c r="K15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="10">
         <f>(L13/L14)*100</f>
         <v>10.822443571232752</v>
       </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
       <c r="P15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="12">
         <f>(Q13/Q14)*100</f>
         <v>8.829363240337381</v>
       </c>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
       <c r="U15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="V15" s="3">
+      <c r="V15" s="10">
         <f>(V13/V14)*100</f>
         <v>7.3412061239731141</v>
       </c>
-      <c r="W15" s="1"/>
-      <c r="X15" s="1"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6787,42 +6796,42 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="9">
         <v>-5.9874099999999997</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="9">
         <f>10^(B3/20)</f>
         <v>0.50191421990127816</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="9">
         <f>C3^2</f>
         <v>0.25191788413910859</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="9">
         <v>9.7491161999999996</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="9">
         <f>10^(G3/20)</f>
         <v>3.072244744665162</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="9">
         <f>H3^2</f>
         <v>9.4386877711227068</v>
       </c>
       <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="9">
         <v>13.1944</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="9">
         <f>10^(L3/20)</f>
         <v>4.5679358894666935</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="9">
         <f>M3^2</f>
         <v>20.866038290277871</v>
       </c>
@@ -6831,42 +6840,42 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="9">
         <v>-47.923389999999998</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="9">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
         <v>4.0163402724472308E-3</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="9">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
         <v>1.6130989184081495E-5</v>
       </c>
       <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="9">
         <v>-25.243649999999999</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="9">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
         <v>5.4678614316365483E-2</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="9">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
         <v>2.9897508635578483E-3</v>
       </c>
       <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="9">
         <v>4.1252880000000003</v>
       </c>
-      <c r="M4" s="2">
+      <c r="M4" s="9">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
         <v>1.6079198623298983</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="9">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
         <v>2.5854062836749989</v>
       </c>
@@ -6875,42 +6884,42 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="9">
         <v>-59.354730000000004</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="9">
         <f t="shared" si="0"/>
         <v>1.0771185368062472E-3</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="9">
         <f t="shared" si="1"/>
         <v>1.1601843423316308E-6</v>
       </c>
       <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="9">
         <v>-40.991669999999999</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="9">
         <f t="shared" si="2"/>
         <v>8.9210608155914466E-3</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="9">
         <f t="shared" si="3"/>
         <v>7.9585326075481128E-5</v>
       </c>
       <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="9">
         <v>-7.5076200000000002</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="9">
         <f t="shared" si="4"/>
         <v>0.42132671767257612</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="9">
         <f t="shared" si="5"/>
         <v>0.17751620302474666</v>
       </c>
@@ -6919,42 +6928,42 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="9">
         <v>-76.521500000000003</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="9">
         <f t="shared" si="0"/>
         <v>1.4925366353760677E-4</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="9">
         <f t="shared" si="1"/>
         <v>2.2276656079397127E-8</v>
       </c>
       <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="9">
         <v>-43.857667999999997</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="9">
         <f t="shared" si="2"/>
         <v>6.4138175255597308E-3</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="9">
         <f t="shared" si="3"/>
         <v>4.1137055251177144E-5</v>
       </c>
       <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="9">
         <v>-3.687646</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="9">
         <f t="shared" si="4"/>
         <v>0.65406016562230995</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="9">
         <f t="shared" si="5"/>
         <v>0.42779470025388355</v>
       </c>
@@ -6963,42 +6972,42 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="9">
         <v>-92.178910000000002</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="9">
         <f t="shared" si="0"/>
         <v>2.4606763772357145E-5</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="9">
         <f t="shared" si="1"/>
         <v>6.054928233485881E-10</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="9">
         <v>-58.687959999999997</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="9">
         <f t="shared" si="2"/>
         <v>1.1630596794038942E-3</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="9">
         <f t="shared" si="3"/>
         <v>1.3527078178550891E-6</v>
       </c>
       <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="9">
         <v>-18.63626</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="9">
         <f t="shared" si="4"/>
         <v>0.11700030664878129</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="9">
         <f t="shared" si="5"/>
         <v>1.3689071755908855E-2</v>
       </c>
@@ -7007,42 +7016,42 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="9">
         <v>-90.704859999999996</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="9">
         <f t="shared" si="0"/>
         <v>2.9157950879776206E-5</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="9">
         <f t="shared" si="1"/>
         <v>8.50186099507442E-10</v>
       </c>
       <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="9">
         <v>-47.371000000000002</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="9">
         <f t="shared" si="2"/>
         <v>4.2800614072157203E-3</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="9">
         <f t="shared" si="3"/>
         <v>1.831892564953741E-5</v>
       </c>
       <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="9">
         <v>-19.527329999999999</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="9">
         <f t="shared" si="4"/>
         <v>0.10559260398339658</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="9">
         <f t="shared" si="5"/>
         <v>1.114979801599442E-2</v>
       </c>
@@ -7051,42 +7060,42 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="9">
         <v>-98.370769999999993</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="9">
         <f t="shared" si="0"/>
         <v>1.2063171440136758E-5</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="9">
         <f t="shared" si="1"/>
         <v>1.4552010519413115E-10</v>
       </c>
       <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="9">
         <v>-55.532060000000001</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="9">
         <f t="shared" si="2"/>
         <v>1.672618900577613E-3</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="9">
         <f t="shared" si="3"/>
         <v>2.7976539865694629E-6</v>
       </c>
       <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="9">
         <v>-41.205199999999998</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="9">
         <f t="shared" si="4"/>
         <v>8.7044232438275235E-3</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="9">
         <f t="shared" si="5"/>
         <v>7.576698400768487E-5</v>
       </c>
@@ -7095,42 +7104,42 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="9">
         <v>-112.23600999999999</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="9">
         <f t="shared" si="0"/>
         <v>2.4445532387858817E-6</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="9">
         <f t="shared" si="1"/>
         <v>5.9758405372585441E-12</v>
       </c>
       <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="9">
         <v>-54.980759999999997</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="9">
         <f t="shared" si="2"/>
         <v>1.7822228192771439E-3</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="9">
         <f t="shared" si="3"/>
         <v>3.1763181775521712E-6</v>
       </c>
       <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="9">
         <v>-27.8599</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="9">
         <f t="shared" si="4"/>
         <v>4.0458054957634139E-2</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="9">
         <f t="shared" si="5"/>
         <v>1.6368542109549444E-3</v>
       </c>
@@ -7139,140 +7148,140 @@
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="9">
         <f>SQRT(SUM(D4:D10)/D3)</f>
         <v>8.2905332850849202E-3</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
       <c r="F11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="9">
         <f>SQRT(SUM(I4:I10)/I3)</f>
         <v>1.8228059874627934E-2</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
       <c r="K11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L11" s="9">
         <f>SQRT(SUM(N4:N10)/N3)</f>
         <v>0.39266633186089883</v>
       </c>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="9">
         <f>B11*100</f>
         <v>0.829053328508492</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
       <c r="F12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="9">
         <f>G11*100</f>
         <v>1.8228059874627933</v>
       </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
       <c r="K12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L12" s="2">
+      <c r="L12" s="9">
         <f>L11*100</f>
         <v>39.266633186089884</v>
       </c>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="9">
         <v>2.5152000000000001</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
       <c r="F13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="9">
         <v>94.245999999999995</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
       <c r="K13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="9">
         <v>244.93</v>
       </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="9">
         <v>78.765000000000001</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
       <c r="F14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="9">
         <v>224.01</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
       <c r="K14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="9">
         <v>388.12</v>
       </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="9">
         <f>(B13/B14)*100</f>
         <v>3.1932965149495334</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
       <c r="F15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="9">
         <f>(G13/G14)*100</f>
         <v>42.072228918351854</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
       <c r="K15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L15" s="1">
+      <c r="L15" s="9">
         <f>(L13/L14)*100</f>
         <v>63.106771101721115</v>
       </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7365,42 +7374,42 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="9">
         <v>-25.274678000000002</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="9">
         <f>10^(B3/20)</f>
         <v>5.4483638159108443E-2</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="9">
         <f>C3^2</f>
         <v>2.9684668270526576E-3</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="9">
         <v>8.9817060000000009</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="9">
         <f>10^(G3/20)</f>
         <v>2.8124531715117249</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="9">
         <f>H3^2</f>
         <v>7.9098928419463599</v>
       </c>
       <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="9">
         <v>19.416899999999998</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="9">
         <f>10^(L3/20)</f>
         <v>9.3507188678557984</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="9">
         <f>M3^2</f>
         <v>87.435943345674431</v>
       </c>
@@ -7409,42 +7418,42 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="9">
         <v>-118.995</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="9">
         <f t="shared" ref="C4:C10" si="0">10^(B4/20)</f>
         <v>1.1226645259802338E-6</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="9">
         <f t="shared" ref="D4:D10" si="1">C4^2</f>
         <v>1.260375637894423E-12</v>
       </c>
       <c r="F4" s="1">
         <v>2</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="9">
         <v>-31.732075999999999</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="9">
         <f t="shared" ref="H4:H10" si="2">10^(G4/20)</f>
         <v>2.5905751783015071E-2</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="9">
         <f t="shared" ref="I4:I10" si="3">H4^2</f>
         <v>6.7110797544318846E-4</v>
       </c>
       <c r="K4" s="1">
         <v>2</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="9">
         <v>-31.116399999999999</v>
       </c>
-      <c r="M4" s="2">
+      <c r="M4" s="9">
         <f t="shared" ref="M4:M10" si="4">10^(L4/20)</f>
         <v>2.7808656012838967E-2</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="9">
         <f t="shared" ref="N4:N10" si="5">M4^2</f>
         <v>7.7332134924040482E-4</v>
       </c>
@@ -7453,42 +7462,42 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="9">
         <v>-29.106104999999999</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="9">
         <f t="shared" si="0"/>
         <v>3.5050542967105115E-2</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="9">
         <f t="shared" si="1"/>
         <v>1.2285405622888819E-3</v>
       </c>
       <c r="F5" s="1">
         <v>3</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="9">
         <v>-14.11999</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="9">
         <f t="shared" si="2"/>
         <v>0.19678885553209666</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="9">
         <f t="shared" si="3"/>
         <v>3.8725853661632406E-2</v>
       </c>
       <c r="K5" s="1">
         <v>3</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="9">
         <v>-5.471406</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="9">
         <f t="shared" si="4"/>
         <v>0.53263499879461385</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="9">
         <f t="shared" si="5"/>
         <v>0.28370004194093829</v>
       </c>
@@ -7497,42 +7506,42 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="9">
         <v>-116.8165</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="9">
         <f t="shared" si="0"/>
         <v>1.4426965724485703E-6</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="9">
         <f t="shared" si="1"/>
         <v>2.0813734001548528E-12</v>
       </c>
       <c r="F6" s="1">
         <v>4</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="9">
         <v>-48.047980000000003</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="9">
         <f t="shared" si="2"/>
         <v>3.9591412835308631E-3</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="9">
         <f t="shared" si="3"/>
         <v>1.5674799702958411E-5</v>
       </c>
       <c r="K6" s="1">
         <v>4</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="9">
         <v>-24.66048</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="9">
         <f t="shared" si="4"/>
         <v>5.8475776834308088E-2</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="9">
         <f t="shared" si="5"/>
         <v>3.4194164763758023E-3</v>
       </c>
@@ -7541,42 +7550,42 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="9">
         <v>-38.732456999999997</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="9">
         <f t="shared" si="0"/>
         <v>1.1571166692173812E-2</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="9">
         <f t="shared" si="1"/>
         <v>1.3389189861807264E-4</v>
       </c>
       <c r="F7" s="1">
         <v>5</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="9">
         <v>-19.348206999999999</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="9">
         <f t="shared" si="2"/>
         <v>0.10779277438543364</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="9">
         <f t="shared" si="3"/>
         <v>1.1619282209708998E-2</v>
       </c>
       <c r="K7" s="1">
         <v>5</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="9">
         <v>-6.723776</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="9">
         <f t="shared" si="4"/>
         <v>0.46111707044912315</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="9">
         <f t="shared" si="5"/>
         <v>0.21262895265958159</v>
       </c>
@@ -7585,42 +7594,42 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="9">
         <v>-114.1957</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="9">
         <f t="shared" si="0"/>
         <v>1.9508101206001143E-6</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="9">
         <f t="shared" si="1"/>
         <v>3.8056601266358327E-12</v>
       </c>
       <c r="F8" s="1">
         <v>6</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="9">
         <v>-60.111530000000002</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="9">
         <f t="shared" si="2"/>
         <v>9.8724172001270314E-4</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="9">
         <f t="shared" si="3"/>
         <v>9.7464621373364063E-7</v>
       </c>
       <c r="K8" s="1">
         <v>6</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="9">
         <v>-33.230699999999999</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="9">
         <f t="shared" si="4"/>
         <v>2.1800426994224943E-2</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="9">
         <f t="shared" si="5"/>
         <v>4.7525861713053157E-4</v>
       </c>
@@ -7629,42 +7638,42 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="9">
         <v>-57.957210000000003</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="9">
         <f t="shared" si="0"/>
         <v>1.2651426594704268E-3</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="9">
         <f t="shared" si="1"/>
         <v>1.6005859488119042E-6</v>
       </c>
       <c r="F9" s="1">
         <v>7</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="9">
         <v>-23.239789999999999</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="9">
         <f t="shared" si="2"/>
         <v>6.8866894619092206E-2</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="9">
         <f t="shared" si="3"/>
         <v>4.7426491744771513E-3</v>
       </c>
       <c r="K9" s="1">
         <v>7</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="9">
         <v>-24.285640000000001</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="9">
         <f t="shared" si="4"/>
         <v>6.1054545130109272E-2</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="9">
         <f t="shared" si="5"/>
         <v>3.7276574810445498E-3</v>
       </c>
@@ -7673,42 +7682,42 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="9">
         <v>-126.1932</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="9">
         <f t="shared" si="0"/>
         <v>4.9016240701903493E-7</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="9">
         <f t="shared" si="1"/>
         <v>2.4025918525469407E-13</v>
       </c>
       <c r="F10" s="1">
         <v>8</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="9">
         <v>-77.061824999999999</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="9">
         <f t="shared" si="2"/>
         <v>1.4025189890889075E-4</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="9">
         <f t="shared" si="3"/>
         <v>1.9670595147549709E-8</v>
       </c>
       <c r="K10" s="1">
         <v>8</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="9">
         <v>-33.091999999999999</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="9">
         <f t="shared" si="4"/>
         <v>2.2151339841371936E-2</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="9">
         <f t="shared" si="5"/>
         <v>4.906818567679517E-4</v>
       </c>
@@ -7717,140 +7726,140 @@
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="9">
         <f>SQRT(SUM(D4:D10)/D3)</f>
         <v>0.67786989575810741</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
       <c r="F11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="9">
         <f>SQRT(SUM(I4:I10)/I3)</f>
         <v>8.3972421687846785E-2</v>
       </c>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
       <c r="K11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L11" s="9">
         <f>SQRT(SUM(N4:N10)/N3)</f>
         <v>7.6013942885339775E-2</v>
       </c>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="9">
         <f>B11*100</f>
         <v>67.786989575810736</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
       <c r="F12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="9">
         <f>G11*100</f>
         <v>8.397242168784679</v>
       </c>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
       <c r="K12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L12" s="2">
+      <c r="L12" s="9">
         <f>L11*100</f>
         <v>7.6013942885339771</v>
       </c>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="9">
         <v>4.3159999999999997E-2</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
       <c r="F13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="9">
         <v>82.626000000000005</v>
       </c>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
       <c r="K13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L13" s="1">
+      <c r="L13" s="9">
         <v>890.77</v>
       </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="9">
         <v>2.4380999999999999</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
       <c r="F14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="9">
         <v>148.26</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
       <c r="K14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="L14" s="1">
+      <c r="L14" s="9">
         <v>251.94</v>
       </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="9">
         <f>(B13/B14)*100</f>
         <v>1.7702309175177393</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
       <c r="F15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="9">
         <f>(G13/G14)*100</f>
         <v>55.730473492513156</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
       <c r="K15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L15" s="1">
+      <c r="L15" s="9">
         <f>(L13/L14)*100</f>
         <v>353.56434071604349</v>
       </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>